<commit_message>
signed off digi GAM
</commit_message>
<xml_diff>
--- a/helper/ins_account_lookup.xlsx
+++ b/helper/ins_account_lookup.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brunsd01/BBC Dropbox/Domi Bruns/Audience Insight/GAM 2025/7. GAM25_calculation/3 DigiGAM/helper/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brunsd01/BBC Dropbox/Domi Bruns/developing/digiGAM/digiGAM/helper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE60954-7673-8740-B45A-627663C24B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522AED3F-0C0B-FE4C-810B-8B2E3C63234A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17820" yWindow="1280" windowWidth="17740" windowHeight="16940" xr2:uid="{8BD58AC2-E357-BC45-B579-2F9F7D382C3C}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" xr2:uid="{8BD58AC2-E357-BC45-B579-2F9F7D382C3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$J$104</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="542">
   <si>
     <t>IG FB Linked ID</t>
   </si>
@@ -713,9 +713,6 @@
     <t>instagram.com/bbc_culture</t>
   </si>
   <si>
-    <t>GNL</t>
-  </si>
-  <si>
     <t>bbc_culture</t>
   </si>
   <si>
@@ -1058,18 +1055,6 @@
     <t>17841405843432881</t>
   </si>
   <si>
-    <t>1048672825173961</t>
-  </si>
-  <si>
-    <t>Antiques Roadshow</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/bbcantiquesroadshow/</t>
-  </si>
-  <si>
-    <t>bbcantiquesroadshow</t>
-  </si>
-  <si>
     <t>17841408230762868</t>
   </si>
   <si>
@@ -1139,15 +1124,6 @@
     <t>176339122382143</t>
   </si>
   <si>
-    <t>Pobol y Cwm</t>
-  </si>
-  <si>
-    <t>https://www.instagram.com/pobol_y_cwm</t>
-  </si>
-  <si>
-    <t>pobol_y_cwm</t>
-  </si>
-  <si>
     <t>17841401623832118</t>
   </si>
   <si>
@@ -1674,6 +1650,21 @@
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t>BNO</t>
+  </si>
+  <si>
+    <t>BNI</t>
+  </si>
+  <si>
+    <t>Pobol y Cwm / Antiques Roadshow</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/pobol_y_cwm or https://www.instagram.com/bbcantiquesroadshow/</t>
+  </si>
+  <si>
+    <t>pobol_y_cwm / bbcantiquesroadshow</t>
   </si>
 </sst>
 </file>
@@ -1767,7 +1758,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1786,9 +1777,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -2128,7 +2116,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBB8FDA3-6C63-BA45-BC17-0CCC0291ABA7}">
-  <dimension ref="A1:J146"/>
+  <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.33203125" style="1" customWidth="1"/>
@@ -2145,19 +2133,19 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>542</v>
+        <v>534</v>
       </c>
       <c r="F1" t="s">
         <v>2</v>
@@ -2166,7 +2154,7 @@
         <v>3</v>
       </c>
       <c r="H1" t="s">
-        <v>543</v>
+        <v>535</v>
       </c>
       <c r="I1" t="s">
         <v>4</v>
@@ -2176,367 +2164,382 @@
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>6</v>
+      <c r="A2" s="1">
+        <v>3958692308</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>411</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>412</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>413</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>217</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>414</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" t="s">
-        <v>6</v>
+        <v>219</v>
+      </c>
+      <c r="J2">
+        <f>A2</f>
+        <v>3958692308</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>14</v>
+      <c r="A3" s="1">
+        <v>7323028146</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>432</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>433</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>434</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>217</v>
       </c>
       <c r="F3" t="s">
-        <v>18</v>
+        <v>435</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3" t="s">
-        <v>13</v>
+        <v>219</v>
+      </c>
+      <c r="J3">
+        <f>A3</f>
+        <v>7323028146</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>20</v>
+      <c r="A4" s="1">
+        <v>35770224198</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>22</v>
+        <v>406</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>407</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>408</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>217</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>409</v>
       </c>
       <c r="H4" t="s">
-        <v>24</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
+        <v>219</v>
+      </c>
+      <c r="I4" t="s">
+        <v>410</v>
+      </c>
+      <c r="J4">
+        <f>A4</f>
+        <v>35770224198</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
-      </c>
-      <c r="J5" t="s">
-        <v>26</v>
+      <c r="A5" s="9">
+        <v>50063441671</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>477</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>478</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="I5" s="9">
+        <v>50063441671</v>
+      </c>
+      <c r="J5" s="9">
+        <v>50063441671</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>33</v>
+      <c r="A6" s="9">
+        <v>59656647810</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
-      <c r="F6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J6" t="s">
-        <v>33</v>
+        <v>473</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>474</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>475</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="I6" s="9">
+        <v>59656647810</v>
+      </c>
+      <c r="J6" s="9">
+        <v>59656647810</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" t="s">
-        <v>39</v>
+      <c r="A7" s="9">
+        <v>60242160822</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>476</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>480</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="I7" s="9">
+        <v>60242160822</v>
+      </c>
+      <c r="J7" s="9">
+        <v>60242160822</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>295</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>296</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>297</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>298</v>
       </c>
       <c r="E8" t="s">
-        <v>50</v>
+        <v>273</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>299</v>
+      </c>
+      <c r="G8" t="s">
+        <v>225</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>275</v>
       </c>
       <c r="J8" t="s">
-        <v>46</v>
+        <v>295</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>52</v>
+        <v>148</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>53</v>
+        <v>149</v>
       </c>
       <c r="C9" t="s">
-        <v>54</v>
+        <v>150</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>151</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>152</v>
       </c>
       <c r="F9" t="s">
-        <v>54</v>
+        <v>153</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>154</v>
       </c>
       <c r="J9" t="s">
-        <v>52</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>59</v>
+        <v>220</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>221</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>222</v>
       </c>
       <c r="D10" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" t="s">
-        <v>62</v>
+        <v>223</v>
       </c>
       <c r="F10" t="s">
-        <v>63</v>
+        <v>224</v>
+      </c>
+      <c r="G10" t="s">
+        <v>225</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>537</v>
       </c>
       <c r="J10" t="s">
-        <v>58</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>65</v>
+      <c r="A11" s="1" t="s">
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="D11" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>48</v>
       </c>
       <c r="H11" t="s">
-        <v>71</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>66</v>
+        <v>51</v>
+      </c>
+      <c r="J11" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>74</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>36</v>
       </c>
       <c r="E12" t="s">
-        <v>76</v>
+        <v>37</v>
       </c>
       <c r="F12" t="s">
-        <v>77</v>
+        <v>35</v>
       </c>
       <c r="H12" t="s">
-        <v>78</v>
+        <v>38</v>
       </c>
       <c r="J12" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>80</v>
+        <v>269</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>270</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>271</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>272</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>273</v>
       </c>
       <c r="F13" t="s">
-        <v>84</v>
+        <v>274</v>
+      </c>
+      <c r="G13" t="s">
+        <v>225</v>
       </c>
       <c r="H13" t="s">
-        <v>85</v>
+        <v>275</v>
       </c>
       <c r="J13" t="s">
-        <v>79</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
-        <v>86</v>
+      <c r="A14" t="s">
+        <v>141</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>143</v>
       </c>
       <c r="D14" t="s">
-        <v>89</v>
+        <v>144</v>
       </c>
       <c r="E14" t="s">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="F14" t="s">
-        <v>91</v>
+        <v>146</v>
       </c>
       <c r="H14" t="s">
-        <v>92</v>
-      </c>
-      <c r="J14" t="s">
-        <v>86</v>
+        <v>147</v>
+      </c>
+      <c r="I14" t="s">
+        <v>141</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>93</v>
+      <c r="A15" s="1" t="s">
+        <v>324</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>94</v>
+        <v>325</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>326</v>
       </c>
       <c r="D15" t="s">
-        <v>95</v>
+        <v>327</v>
       </c>
       <c r="E15" t="s">
-        <v>24</v>
+        <v>217</v>
       </c>
       <c r="F15" t="s">
-        <v>96</v>
+        <v>326</v>
       </c>
       <c r="H15" t="s">
-        <v>24</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>93</v>
+        <v>219</v>
+      </c>
+      <c r="J15" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -2566,292 +2569,302 @@
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>104</v>
+      <c r="A17" t="s">
+        <v>521</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>522</v>
       </c>
       <c r="C17" t="s">
-        <v>105</v>
-      </c>
-      <c r="D17" t="s">
-        <v>106</v>
-      </c>
-      <c r="E17" t="s">
-        <v>107</v>
+        <v>523</v>
       </c>
       <c r="F17" t="s">
-        <v>105</v>
+        <v>524</v>
+      </c>
+      <c r="G17" t="s">
+        <v>536</v>
       </c>
       <c r="H17" t="s">
-        <v>108</v>
-      </c>
-      <c r="J17" t="s">
-        <v>103</v>
+        <v>537</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>109</v>
+        <v>427</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>111</v>
+        <v>428</v>
+      </c>
+      <c r="C18" t="s">
+        <v>429</v>
       </c>
       <c r="D18" t="s">
-        <v>112</v>
+        <v>430</v>
       </c>
       <c r="E18" t="s">
-        <v>113</v>
+        <v>273</v>
       </c>
       <c r="F18" t="s">
-        <v>114</v>
+        <v>431</v>
+      </c>
+      <c r="G18" t="s">
+        <v>536</v>
       </c>
       <c r="H18" t="s">
-        <v>115</v>
-      </c>
-      <c r="J18" t="s">
-        <v>109</v>
+        <v>275</v>
+      </c>
+      <c r="I18" t="s">
+        <v>427</v>
+      </c>
+      <c r="J18" t="str">
+        <f>A18</f>
+        <v>17841400778089100</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>117</v>
+        <v>26</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>119</v>
+        <v>29</v>
       </c>
       <c r="E19" t="s">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>31</v>
       </c>
       <c r="H19" t="s">
-        <v>122</v>
+        <v>32</v>
       </c>
       <c r="J19" t="s">
-        <v>116</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>123</v>
+        <v>161</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>124</v>
+        <v>162</v>
       </c>
       <c r="C20" t="s">
-        <v>125</v>
+        <v>163</v>
       </c>
       <c r="D20" t="s">
-        <v>126</v>
+        <v>164</v>
       </c>
       <c r="E20" t="s">
-        <v>127</v>
+        <v>165</v>
       </c>
       <c r="F20" t="s">
-        <v>125</v>
+        <v>163</v>
       </c>
       <c r="H20" t="s">
-        <v>128</v>
+        <v>166</v>
       </c>
       <c r="J20" t="s">
-        <v>123</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>130</v>
+        <v>371</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>372</v>
       </c>
       <c r="C21" t="s">
-        <v>131</v>
+        <v>373</v>
       </c>
       <c r="D21" t="s">
-        <v>132</v>
+        <v>374</v>
       </c>
       <c r="E21" t="s">
-        <v>133</v>
+        <v>273</v>
       </c>
       <c r="F21" t="s">
-        <v>131</v>
+        <v>375</v>
+      </c>
+      <c r="G21" t="s">
+        <v>536</v>
       </c>
       <c r="H21" t="s">
-        <v>134</v>
+        <v>275</v>
       </c>
       <c r="J21" t="s">
-        <v>129</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>135</v>
+      <c r="A22" t="s">
+        <v>180</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>136</v>
+        <v>181</v>
       </c>
       <c r="C22" t="s">
-        <v>137</v>
+        <v>182</v>
       </c>
       <c r="D22" t="s">
-        <v>138</v>
+        <v>183</v>
       </c>
       <c r="E22" t="s">
-        <v>139</v>
+        <v>184</v>
       </c>
       <c r="F22" t="s">
-        <v>137</v>
+        <v>185</v>
       </c>
       <c r="H22" t="s">
-        <v>140</v>
-      </c>
-      <c r="J22" t="s">
-        <v>135</v>
+        <v>186</v>
+      </c>
+      <c r="I22" t="s">
+        <v>180</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>141</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>142</v>
+      <c r="A23" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>281</v>
       </c>
       <c r="C23" t="s">
-        <v>143</v>
+        <v>282</v>
       </c>
       <c r="D23" t="s">
-        <v>144</v>
+        <v>283</v>
       </c>
       <c r="E23" t="s">
-        <v>145</v>
+        <v>273</v>
       </c>
       <c r="F23" t="s">
-        <v>146</v>
+        <v>284</v>
+      </c>
+      <c r="G23" t="s">
+        <v>225</v>
       </c>
       <c r="H23" t="s">
-        <v>147</v>
-      </c>
-      <c r="I23" t="s">
-        <v>141</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>142</v>
+        <v>275</v>
+      </c>
+      <c r="J23" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>148</v>
+        <v>201</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>149</v>
+        <v>202</v>
       </c>
       <c r="C24" t="s">
-        <v>150</v>
+        <v>203</v>
       </c>
       <c r="D24" t="s">
-        <v>151</v>
+        <v>204</v>
       </c>
       <c r="E24" t="s">
-        <v>152</v>
+        <v>205</v>
       </c>
       <c r="F24" t="s">
-        <v>153</v>
+        <v>206</v>
       </c>
       <c r="H24" t="s">
-        <v>154</v>
+        <v>207</v>
       </c>
       <c r="J24" t="s">
-        <v>148</v>
+        <v>201</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>155</v>
+        <v>236</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>156</v>
+        <v>237</v>
       </c>
       <c r="C25" t="s">
-        <v>157</v>
+        <v>238</v>
       </c>
       <c r="D25" t="s">
-        <v>158</v>
+        <v>239</v>
       </c>
       <c r="E25" t="s">
-        <v>159</v>
+        <v>240</v>
       </c>
       <c r="F25" t="s">
-        <v>157</v>
+        <v>241</v>
       </c>
       <c r="H25" t="s">
-        <v>160</v>
+        <v>242</v>
       </c>
       <c r="J25" t="s">
-        <v>155</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>162</v>
+        <v>366</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>367</v>
       </c>
       <c r="C26" t="s">
-        <v>163</v>
+        <v>368</v>
       </c>
       <c r="D26" t="s">
-        <v>164</v>
+        <v>369</v>
       </c>
       <c r="E26" t="s">
-        <v>165</v>
+        <v>273</v>
       </c>
       <c r="F26" t="s">
-        <v>163</v>
+        <v>370</v>
+      </c>
+      <c r="G26" t="s">
+        <v>536</v>
       </c>
       <c r="H26" t="s">
-        <v>166</v>
+        <v>275</v>
       </c>
       <c r="J26" t="s">
-        <v>161</v>
+        <v>366</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A27" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="C27" t="s">
-        <v>169</v>
-      </c>
-      <c r="D27" t="s">
-        <v>170</v>
-      </c>
-      <c r="E27" t="s">
-        <v>171</v>
+      <c r="A27" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>394</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>395</v>
       </c>
       <c r="F27" t="s">
-        <v>169</v>
+        <v>394</v>
+      </c>
+      <c r="G27" t="s">
+        <v>536</v>
       </c>
       <c r="H27" t="s">
-        <v>172</v>
-      </c>
-      <c r="J27" t="s">
-        <v>167</v>
+        <v>537</v>
+      </c>
+      <c r="J27">
+        <v>349617059</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
@@ -2881,110 +2894,110 @@
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>180</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>181</v>
+      <c r="A29" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C29" t="s">
-        <v>182</v>
+        <v>41</v>
       </c>
       <c r="D29" t="s">
-        <v>183</v>
+        <v>42</v>
       </c>
       <c r="E29" t="s">
-        <v>184</v>
+        <v>43</v>
       </c>
       <c r="F29" t="s">
-        <v>185</v>
+        <v>44</v>
       </c>
       <c r="H29" t="s">
-        <v>186</v>
-      </c>
-      <c r="I29" t="s">
-        <v>180</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>181</v>
+        <v>45</v>
+      </c>
+      <c r="J29" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>187</v>
+        <v>52</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>188</v>
+        <v>53</v>
       </c>
       <c r="C30" t="s">
-        <v>189</v>
+        <v>54</v>
       </c>
       <c r="D30" t="s">
-        <v>190</v>
+        <v>55</v>
       </c>
       <c r="E30" t="s">
-        <v>191</v>
+        <v>56</v>
       </c>
       <c r="F30" t="s">
-        <v>192</v>
+        <v>54</v>
       </c>
       <c r="H30" t="s">
-        <v>193</v>
+        <v>57</v>
       </c>
       <c r="J30" t="s">
-        <v>187</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>194</v>
+        <v>231</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>195</v>
+        <v>232</v>
       </c>
       <c r="C31" t="s">
-        <v>196</v>
+        <v>233</v>
       </c>
       <c r="D31" t="s">
-        <v>197</v>
-      </c>
-      <c r="E31" t="s">
-        <v>198</v>
+        <v>234</v>
       </c>
       <c r="F31" t="s">
-        <v>199</v>
+        <v>235</v>
+      </c>
+      <c r="G31" t="s">
+        <v>225</v>
       </c>
       <c r="H31" t="s">
-        <v>200</v>
+        <v>537</v>
       </c>
       <c r="J31" t="s">
-        <v>194</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>201</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>202</v>
+        <v>361</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>362</v>
       </c>
       <c r="C32" t="s">
-        <v>203</v>
+        <v>363</v>
       </c>
       <c r="D32" t="s">
-        <v>204</v>
+        <v>364</v>
       </c>
       <c r="E32" t="s">
-        <v>205</v>
+        <v>273</v>
       </c>
       <c r="F32" t="s">
-        <v>206</v>
+        <v>365</v>
+      </c>
+      <c r="G32" t="s">
+        <v>536</v>
       </c>
       <c r="H32" t="s">
-        <v>207</v>
+        <v>275</v>
       </c>
       <c r="J32" t="s">
-        <v>201</v>
+        <v>361</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
@@ -3015,1902 +3028,1831 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>213</v>
+        <v>187</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>215</v>
+        <v>188</v>
+      </c>
+      <c r="C34" t="s">
+        <v>189</v>
       </c>
       <c r="D34" t="s">
-        <v>216</v>
+        <v>190</v>
       </c>
       <c r="E34" t="s">
-        <v>217</v>
+        <v>191</v>
       </c>
       <c r="F34" t="s">
-        <v>218</v>
+        <v>192</v>
       </c>
       <c r="H34" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="J34" t="s">
-        <v>213</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>221</v>
+      <c r="A35" s="6" t="s">
+        <v>531</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>343</v>
       </c>
       <c r="C35" t="s">
-        <v>222</v>
+        <v>344</v>
       </c>
       <c r="D35" t="s">
-        <v>223</v>
+        <v>345</v>
       </c>
       <c r="E35" t="s">
-        <v>224</v>
+        <v>273</v>
       </c>
       <c r="F35" t="s">
-        <v>225</v>
+        <v>346</v>
       </c>
       <c r="G35" t="s">
-        <v>226</v>
+        <v>536</v>
       </c>
       <c r="H35" t="s">
-        <v>224</v>
-      </c>
-      <c r="J35" t="s">
-        <v>220</v>
+        <v>275</v>
+      </c>
+      <c r="J35" s="7">
+        <v>1397240097</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>228</v>
+        <v>58</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="C36" t="s">
-        <v>229</v>
+        <v>60</v>
       </c>
       <c r="D36" t="s">
-        <v>230</v>
+        <v>61</v>
       </c>
       <c r="E36" t="s">
-        <v>224</v>
+        <v>62</v>
       </c>
       <c r="F36" t="s">
-        <v>231</v>
-      </c>
-      <c r="G36" t="s">
-        <v>226</v>
+        <v>63</v>
       </c>
       <c r="H36" t="s">
-        <v>224</v>
+        <v>64</v>
       </c>
       <c r="J36" t="s">
-        <v>227</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>233</v>
+        <v>347</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>348</v>
       </c>
       <c r="C37" t="s">
-        <v>234</v>
+        <v>349</v>
       </c>
       <c r="D37" t="s">
-        <v>235</v>
+        <v>350</v>
       </c>
       <c r="E37" t="s">
-        <v>224</v>
+        <v>273</v>
       </c>
       <c r="F37" t="s">
-        <v>236</v>
+        <v>349</v>
       </c>
       <c r="G37" t="s">
-        <v>226</v>
+        <v>536</v>
       </c>
       <c r="H37" t="s">
-        <v>224</v>
+        <v>275</v>
       </c>
       <c r="J37" t="s">
-        <v>232</v>
+        <v>347</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="C38" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="D38" t="s">
-        <v>240</v>
-      </c>
-      <c r="E38" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="F38" t="s">
-        <v>242</v>
+        <v>230</v>
+      </c>
+      <c r="G38" t="s">
+        <v>225</v>
       </c>
       <c r="H38" t="s">
-        <v>243</v>
+        <v>537</v>
       </c>
       <c r="J38" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>244</v>
+        <v>6</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>245</v>
+        <v>7</v>
       </c>
       <c r="C39" t="s">
-        <v>246</v>
+        <v>8</v>
       </c>
       <c r="D39" t="s">
-        <v>247</v>
+        <v>9</v>
       </c>
       <c r="E39" t="s">
-        <v>248</v>
+        <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>249</v>
+        <v>11</v>
       </c>
       <c r="H39" t="s">
-        <v>250</v>
+        <v>12</v>
       </c>
       <c r="J39" t="s">
-        <v>244</v>
+        <v>6</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>251</v>
+        <v>86</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>252</v>
+        <v>87</v>
       </c>
       <c r="C40" t="s">
-        <v>253</v>
+        <v>88</v>
       </c>
       <c r="D40" t="s">
-        <v>254</v>
+        <v>89</v>
       </c>
       <c r="E40" t="s">
-        <v>255</v>
+        <v>90</v>
       </c>
       <c r="F40" t="s">
-        <v>256</v>
+        <v>91</v>
       </c>
       <c r="H40" t="s">
-        <v>257</v>
+        <v>92</v>
       </c>
       <c r="J40" t="s">
-        <v>251</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>258</v>
+        <v>213</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="C41" t="s">
-        <v>260</v>
+        <v>214</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>215</v>
       </c>
       <c r="D41" t="s">
-        <v>261</v>
+        <v>216</v>
       </c>
       <c r="E41" t="s">
-        <v>262</v>
+        <v>217</v>
       </c>
       <c r="F41" t="s">
-        <v>263</v>
+        <v>218</v>
       </c>
       <c r="H41" t="s">
-        <v>264</v>
+        <v>219</v>
       </c>
       <c r="J41" t="s">
-        <v>258</v>
+        <v>213</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>265</v>
+        <v>194</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>266</v>
+        <v>195</v>
       </c>
       <c r="C42" t="s">
-        <v>267</v>
+        <v>196</v>
       </c>
       <c r="D42" t="s">
-        <v>268</v>
+        <v>197</v>
       </c>
       <c r="E42" t="s">
-        <v>224</v>
+        <v>198</v>
       </c>
       <c r="F42" t="s">
-        <v>269</v>
-      </c>
-      <c r="G42" t="s">
-        <v>544</v>
+        <v>199</v>
       </c>
       <c r="H42" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="J42" t="s">
-        <v>265</v>
+        <v>194</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C43" t="s">
-        <v>272</v>
+        <v>319</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>321</v>
       </c>
       <c r="D43" t="s">
-        <v>273</v>
+        <v>322</v>
       </c>
       <c r="E43" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="F43" t="s">
-        <v>275</v>
-      </c>
-      <c r="G43" t="s">
-        <v>226</v>
+        <v>323</v>
       </c>
       <c r="H43" t="s">
-        <v>276</v>
+        <v>219</v>
       </c>
       <c r="J43" t="s">
-        <v>270</v>
+        <v>319</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="C44" t="s">
-        <v>279</v>
+        <v>305</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>307</v>
       </c>
       <c r="D44" t="s">
-        <v>280</v>
+        <v>308</v>
       </c>
       <c r="E44" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="F44" t="s">
-        <v>279</v>
-      </c>
-      <c r="G44" t="s">
-        <v>226</v>
+        <v>307</v>
       </c>
       <c r="H44" t="s">
-        <v>276</v>
+        <v>219</v>
       </c>
       <c r="J44" t="s">
-        <v>277</v>
+        <v>305</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>282</v>
+        <v>167</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>168</v>
       </c>
       <c r="C45" t="s">
-        <v>283</v>
+        <v>169</v>
       </c>
       <c r="D45" t="s">
-        <v>284</v>
+        <v>170</v>
       </c>
       <c r="E45" t="s">
-        <v>274</v>
+        <v>171</v>
       </c>
       <c r="F45" t="s">
-        <v>285</v>
-      </c>
-      <c r="G45" t="s">
-        <v>226</v>
+        <v>169</v>
       </c>
       <c r="H45" t="s">
-        <v>276</v>
+        <v>172</v>
       </c>
       <c r="J45" t="s">
-        <v>281</v>
+        <v>167</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>287</v>
+        <v>13</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="C46" t="s">
-        <v>288</v>
+        <v>15</v>
       </c>
       <c r="D46" t="s">
-        <v>289</v>
+        <v>16</v>
       </c>
       <c r="E46" t="s">
-        <v>274</v>
+        <v>17</v>
       </c>
       <c r="F46" t="s">
-        <v>290</v>
-      </c>
-      <c r="G46" t="s">
-        <v>226</v>
+        <v>18</v>
       </c>
       <c r="H46" t="s">
-        <v>276</v>
+        <v>19</v>
       </c>
       <c r="J46" t="s">
-        <v>286</v>
+        <v>13</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>292</v>
+        <v>155</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>156</v>
       </c>
       <c r="C47" t="s">
-        <v>293</v>
+        <v>157</v>
       </c>
       <c r="D47" t="s">
-        <v>294</v>
+        <v>158</v>
       </c>
       <c r="E47" t="s">
-        <v>274</v>
+        <v>159</v>
       </c>
       <c r="F47" t="s">
-        <v>295</v>
-      </c>
-      <c r="G47" t="s">
-        <v>226</v>
+        <v>157</v>
       </c>
       <c r="H47" t="s">
-        <v>276</v>
+        <v>160</v>
       </c>
       <c r="J47" t="s">
-        <v>291</v>
+        <v>155</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>297</v>
+        <v>20</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>21</v>
       </c>
       <c r="C48" t="s">
-        <v>298</v>
+        <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>299</v>
+        <v>23</v>
       </c>
       <c r="E48" t="s">
-        <v>274</v>
+        <v>24</v>
       </c>
       <c r="F48" t="s">
-        <v>300</v>
-      </c>
-      <c r="G48" t="s">
-        <v>226</v>
+        <v>25</v>
       </c>
       <c r="H48" t="s">
-        <v>276</v>
+        <v>24</v>
       </c>
       <c r="J48" t="s">
-        <v>296</v>
+        <v>20</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>302</v>
+      <c r="A49" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>315</v>
       </c>
       <c r="C49" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="D49" t="s">
-        <v>304</v>
+        <v>317</v>
       </c>
       <c r="E49" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="F49" t="s">
-        <v>305</v>
-      </c>
-      <c r="G49" t="s">
-        <v>226</v>
+        <v>318</v>
       </c>
       <c r="H49" t="s">
-        <v>276</v>
-      </c>
-      <c r="J49" t="s">
-        <v>301</v>
+        <v>219</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
-        <v>306</v>
+      <c r="A50" s="2" t="s">
+        <v>65</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>308</v>
+        <v>66</v>
+      </c>
+      <c r="C50" t="s">
+        <v>67</v>
       </c>
       <c r="D50" t="s">
-        <v>309</v>
+        <v>68</v>
       </c>
       <c r="E50" t="s">
-        <v>217</v>
+        <v>69</v>
       </c>
       <c r="F50" t="s">
-        <v>308</v>
+        <v>70</v>
       </c>
       <c r="H50" t="s">
-        <v>219</v>
-      </c>
-      <c r="J50" t="s">
-        <v>306</v>
+        <v>71</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>310</v>
+        <v>72</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>311</v>
+        <v>73</v>
       </c>
       <c r="C51" t="s">
-        <v>312</v>
+        <v>74</v>
       </c>
       <c r="D51" t="s">
-        <v>313</v>
+        <v>75</v>
       </c>
       <c r="E51" t="s">
-        <v>217</v>
+        <v>76</v>
       </c>
       <c r="F51" t="s">
-        <v>314</v>
+        <v>77</v>
       </c>
       <c r="H51" t="s">
-        <v>219</v>
+        <v>78</v>
       </c>
       <c r="J51" t="s">
-        <v>310</v>
+        <v>72</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A52" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>316</v>
+      <c r="A52" s="1" t="s">
+        <v>528</v>
       </c>
       <c r="C52" t="s">
-        <v>317</v>
-      </c>
-      <c r="D52" t="s">
-        <v>318</v>
-      </c>
-      <c r="E52" t="s">
-        <v>217</v>
+        <v>529</v>
       </c>
       <c r="F52" t="s">
-        <v>319</v>
+        <v>530</v>
       </c>
       <c r="H52" t="s">
         <v>219</v>
       </c>
-      <c r="J52" s="2" t="s">
-        <v>315</v>
-      </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>320</v>
+        <v>436</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>321</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>322</v>
+        <v>437</v>
+      </c>
+      <c r="C53" t="s">
+        <v>438</v>
       </c>
       <c r="D53" t="s">
-        <v>323</v>
-      </c>
-      <c r="E53" t="s">
-        <v>217</v>
+        <v>439</v>
       </c>
       <c r="F53" t="s">
-        <v>324</v>
+        <v>440</v>
+      </c>
+      <c r="G53" t="s">
+        <v>225</v>
       </c>
       <c r="H53" t="s">
-        <v>219</v>
-      </c>
-      <c r="J53" t="s">
-        <v>320</v>
+        <v>538</v>
+      </c>
+      <c r="I53" t="s">
+        <v>436</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>325</v>
+        <v>79</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>326</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>327</v>
+        <v>80</v>
+      </c>
+      <c r="C54" t="s">
+        <v>81</v>
       </c>
       <c r="D54" t="s">
-        <v>328</v>
+        <v>82</v>
       </c>
       <c r="E54" t="s">
-        <v>217</v>
+        <v>83</v>
       </c>
       <c r="F54" t="s">
-        <v>327</v>
+        <v>84</v>
       </c>
       <c r="H54" t="s">
-        <v>219</v>
+        <v>85</v>
       </c>
       <c r="J54" t="s">
-        <v>325</v>
+        <v>79</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
-        <v>329</v>
+        <v>129</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>330</v>
-      </c>
-      <c r="C55" s="5" t="s">
-        <v>331</v>
+        <v>130</v>
+      </c>
+      <c r="C55" t="s">
+        <v>131</v>
       </c>
       <c r="D55" t="s">
-        <v>332</v>
+        <v>132</v>
       </c>
       <c r="E55" t="s">
-        <v>217</v>
+        <v>133</v>
       </c>
       <c r="F55" t="s">
-        <v>333</v>
+        <v>131</v>
       </c>
       <c r="H55" t="s">
-        <v>219</v>
+        <v>134</v>
       </c>
       <c r="J55" t="s">
-        <v>329</v>
+        <v>129</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>335</v>
+        <v>103</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>104</v>
       </c>
       <c r="C56" t="s">
-        <v>336</v>
+        <v>105</v>
       </c>
       <c r="D56" t="s">
-        <v>337</v>
+        <v>106</v>
       </c>
       <c r="E56" t="s">
-        <v>274</v>
+        <v>107</v>
       </c>
       <c r="F56" t="s">
-        <v>336</v>
-      </c>
-      <c r="G56" t="s">
-        <v>544</v>
+        <v>105</v>
       </c>
       <c r="H56" t="s">
-        <v>276</v>
+        <v>108</v>
       </c>
       <c r="J56" t="s">
-        <v>334</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
-        <v>338</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>339</v>
+        <v>135</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="C57" t="s">
-        <v>340</v>
+        <v>137</v>
       </c>
       <c r="D57" t="s">
-        <v>341</v>
+        <v>138</v>
       </c>
       <c r="E57" t="s">
-        <v>274</v>
+        <v>139</v>
       </c>
       <c r="F57" t="s">
-        <v>342</v>
-      </c>
-      <c r="G57" t="s">
-        <v>544</v>
+        <v>137</v>
       </c>
       <c r="H57" t="s">
-        <v>276</v>
+        <v>140</v>
       </c>
       <c r="J57" t="s">
-        <v>338</v>
+        <v>135</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>344</v>
+        <v>116</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="C58" t="s">
-        <v>345</v>
+        <v>118</v>
       </c>
       <c r="D58" t="s">
-        <v>346</v>
+        <v>119</v>
       </c>
       <c r="E58" t="s">
-        <v>274</v>
+        <v>120</v>
       </c>
       <c r="F58" t="s">
-        <v>347</v>
-      </c>
-      <c r="G58" t="s">
-        <v>544</v>
+        <v>121</v>
       </c>
       <c r="H58" t="s">
-        <v>276</v>
+        <v>122</v>
       </c>
       <c r="J58" t="s">
-        <v>343</v>
+        <v>116</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A59" s="6" t="s">
-        <v>539</v>
+      <c r="A59" s="1" t="s">
+        <v>285</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>348</v>
+        <v>286</v>
       </c>
       <c r="C59" t="s">
-        <v>349</v>
+        <v>287</v>
       </c>
       <c r="D59" t="s">
-        <v>350</v>
+        <v>288</v>
       </c>
       <c r="E59" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F59" t="s">
-        <v>351</v>
+        <v>289</v>
       </c>
       <c r="G59" t="s">
-        <v>544</v>
+        <v>225</v>
       </c>
       <c r="H59" t="s">
-        <v>276</v>
-      </c>
-      <c r="J59" s="7">
-        <v>1397240097</v>
+        <v>275</v>
+      </c>
+      <c r="J59" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="B60" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="B60" s="3" t="s">
+      <c r="C60" t="s">
         <v>353</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>354</v>
       </c>
-      <c r="D60" t="s">
+      <c r="E60" t="s">
+        <v>273</v>
+      </c>
+      <c r="F60" t="s">
         <v>355</v>
       </c>
-      <c r="E60" t="s">
-        <v>274</v>
-      </c>
-      <c r="F60" t="s">
-        <v>354</v>
-      </c>
       <c r="G60" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="H60" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J60" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="B61" s="3" t="s">
-        <v>357</v>
-      </c>
-      <c r="C61" t="s">
-        <v>358</v>
+        <v>328</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>330</v>
       </c>
       <c r="D61" t="s">
-        <v>359</v>
+        <v>331</v>
       </c>
       <c r="E61" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="F61" t="s">
-        <v>360</v>
-      </c>
-      <c r="G61" t="s">
-        <v>544</v>
+        <v>332</v>
       </c>
       <c r="H61" t="s">
-        <v>276</v>
+        <v>219</v>
       </c>
       <c r="J61" t="s">
-        <v>356</v>
+        <v>328</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>362</v>
+        <v>123</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>124</v>
       </c>
       <c r="C62" t="s">
-        <v>363</v>
+        <v>125</v>
       </c>
       <c r="D62" t="s">
-        <v>364</v>
+        <v>126</v>
       </c>
       <c r="E62" t="s">
-        <v>274</v>
+        <v>127</v>
       </c>
       <c r="F62" t="s">
-        <v>363</v>
-      </c>
-      <c r="G62" t="s">
-        <v>544</v>
+        <v>125</v>
       </c>
       <c r="H62" t="s">
-        <v>276</v>
+        <v>128</v>
       </c>
       <c r="J62" t="s">
-        <v>361</v>
+        <v>123</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="C63" t="s">
-        <v>366</v>
+        <v>539</v>
       </c>
       <c r="D63" t="s">
-        <v>367</v>
+        <v>540</v>
       </c>
       <c r="E63" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F63" t="s">
-        <v>368</v>
+        <v>541</v>
       </c>
       <c r="G63" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="H63" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J63" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
-        <v>369</v>
+        <v>290</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>370</v>
+        <v>291</v>
       </c>
       <c r="C64" t="s">
-        <v>371</v>
+        <v>292</v>
       </c>
       <c r="D64" t="s">
-        <v>372</v>
+        <v>293</v>
       </c>
       <c r="E64" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F64" t="s">
-        <v>373</v>
+        <v>294</v>
       </c>
       <c r="G64" t="s">
-        <v>544</v>
+        <v>225</v>
       </c>
       <c r="H64" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J64" t="s">
-        <v>369</v>
+        <v>290</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
-        <v>374</v>
-      </c>
-      <c r="B65" s="3" t="s">
-        <v>375</v>
-      </c>
-      <c r="C65" t="s">
-        <v>376</v>
+        <v>109</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>111</v>
       </c>
       <c r="D65" t="s">
-        <v>377</v>
+        <v>112</v>
       </c>
       <c r="E65" t="s">
-        <v>274</v>
+        <v>113</v>
       </c>
       <c r="F65" t="s">
-        <v>378</v>
-      </c>
-      <c r="G65" t="s">
-        <v>544</v>
+        <v>114</v>
       </c>
       <c r="H65" t="s">
-        <v>276</v>
+        <v>115</v>
       </c>
       <c r="J65" t="s">
-        <v>374</v>
+        <v>109</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
-        <v>379</v>
-      </c>
-      <c r="B66" s="3" t="s">
-        <v>380</v>
+        <v>309</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>310</v>
       </c>
       <c r="C66" t="s">
-        <v>381</v>
+        <v>311</v>
       </c>
       <c r="D66" t="s">
-        <v>382</v>
+        <v>312</v>
       </c>
       <c r="E66" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="F66" t="s">
-        <v>383</v>
-      </c>
-      <c r="G66" t="s">
-        <v>544</v>
+        <v>313</v>
       </c>
       <c r="H66" t="s">
-        <v>276</v>
+        <v>219</v>
       </c>
       <c r="J66" t="s">
-        <v>379</v>
+        <v>309</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
-        <v>384</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>385</v>
+        <v>257</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>258</v>
       </c>
       <c r="C67" t="s">
-        <v>386</v>
+        <v>259</v>
       </c>
       <c r="D67" t="s">
-        <v>387</v>
+        <v>260</v>
       </c>
       <c r="E67" t="s">
-        <v>274</v>
+        <v>261</v>
       </c>
       <c r="F67" t="s">
-        <v>386</v>
-      </c>
-      <c r="G67" t="s">
-        <v>544</v>
+        <v>262</v>
       </c>
       <c r="H67" t="s">
-        <v>276</v>
+        <v>263</v>
       </c>
       <c r="J67" t="s">
-        <v>384</v>
+        <v>257</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
-        <v>388</v>
+        <v>250</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>389</v>
-      </c>
-      <c r="C68" s="5" t="s">
-        <v>390</v>
+        <v>251</v>
+      </c>
+      <c r="C68" t="s">
+        <v>252</v>
       </c>
       <c r="D68" t="s">
-        <v>391</v>
+        <v>253</v>
       </c>
       <c r="E68" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
       <c r="F68" t="s">
-        <v>390</v>
+        <v>255</v>
       </c>
       <c r="H68" t="s">
-        <v>219</v>
+        <v>256</v>
       </c>
       <c r="J68" t="s">
-        <v>388</v>
+        <v>250</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>393</v>
+        <v>385</v>
       </c>
       <c r="C69" s="5" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="D69" t="s">
-        <v>395</v>
+        <v>387</v>
       </c>
       <c r="E69" t="s">
         <v>217</v>
       </c>
       <c r="F69" t="s">
-        <v>394</v>
+        <v>386</v>
       </c>
       <c r="H69" t="s">
         <v>219</v>
       </c>
       <c r="J69" t="s">
-        <v>392</v>
+        <v>384</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
-        <v>396</v>
+        <v>243</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>397</v>
-      </c>
-      <c r="C70" s="5" t="s">
-        <v>398</v>
+        <v>244</v>
+      </c>
+      <c r="C70" t="s">
+        <v>245</v>
       </c>
       <c r="D70" t="s">
-        <v>399</v>
+        <v>246</v>
       </c>
       <c r="E70" t="s">
-        <v>217</v>
+        <v>247</v>
       </c>
       <c r="F70" t="s">
-        <v>398</v>
+        <v>248</v>
       </c>
       <c r="H70" t="s">
-        <v>219</v>
+        <v>249</v>
       </c>
       <c r="J70" t="s">
-        <v>396</v>
+        <v>243</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A71" s="2" t="s">
-        <v>400</v>
+      <c r="A71" s="1" t="s">
+        <v>338</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>401</v>
-      </c>
-      <c r="C71" s="5" t="s">
-        <v>402</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>403</v>
+        <v>339</v>
+      </c>
+      <c r="C71" t="s">
+        <v>340</v>
+      </c>
+      <c r="D71" t="s">
+        <v>341</v>
       </c>
       <c r="E71" t="s">
-        <v>224</v>
+        <v>273</v>
       </c>
       <c r="F71" t="s">
-        <v>402</v>
+        <v>342</v>
       </c>
       <c r="G71" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="H71" t="s">
-        <v>224</v>
-      </c>
-      <c r="J71">
-        <v>349617059</v>
+        <v>275</v>
+      </c>
+      <c r="J71" t="s">
+        <v>338</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>405</v>
+        <v>276</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>277</v>
       </c>
       <c r="C72" t="s">
-        <v>406</v>
+        <v>278</v>
       </c>
       <c r="D72" t="s">
-        <v>407</v>
+        <v>279</v>
       </c>
       <c r="E72" t="s">
-        <v>224</v>
+        <v>273</v>
       </c>
       <c r="F72" t="s">
-        <v>408</v>
+        <v>278</v>
       </c>
       <c r="G72" t="s">
-        <v>544</v>
+        <v>225</v>
       </c>
       <c r="H72" t="s">
-        <v>224</v>
-      </c>
-      <c r="J72" t="str">
-        <f>A72</f>
-        <v>17841428945200784</v>
+        <v>275</v>
+      </c>
+      <c r="J72" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>410</v>
+        <v>300</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>301</v>
       </c>
       <c r="C73" t="s">
-        <v>411</v>
+        <v>302</v>
       </c>
       <c r="D73" t="s">
-        <v>412</v>
+        <v>303</v>
       </c>
       <c r="E73" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="F73" t="s">
-        <v>413</v>
+        <v>304</v>
+      </c>
+      <c r="G73" t="s">
+        <v>225</v>
       </c>
       <c r="H73" t="s">
-        <v>219</v>
-      </c>
-      <c r="J73" t="str">
-        <f t="shared" ref="J73:J79" si="0">A73</f>
-        <v>17841435108167586</v>
+        <v>275</v>
+      </c>
+      <c r="J73" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A74" s="1">
-        <v>35770224198</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="C74" s="5" t="s">
-        <v>415</v>
+      <c r="A74" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="B74" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="C74" t="s">
+        <v>335</v>
       </c>
       <c r="D74" t="s">
-        <v>416</v>
+        <v>336</v>
       </c>
       <c r="E74" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="F74" t="s">
-        <v>417</v>
+        <v>335</v>
+      </c>
+      <c r="G74" t="s">
+        <v>536</v>
       </c>
       <c r="H74" t="s">
-        <v>219</v>
-      </c>
-      <c r="I74" t="s">
-        <v>418</v>
-      </c>
-      <c r="J74">
-        <f t="shared" si="0"/>
-        <v>35770224198</v>
+        <v>275</v>
+      </c>
+      <c r="J74" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A75" s="1">
-        <v>3958692308</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>419</v>
-      </c>
-      <c r="C75" t="s">
-        <v>420</v>
+      <c r="A75" s="1" t="s">
+        <v>461</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>462</v>
       </c>
       <c r="D75" t="s">
-        <v>421</v>
+        <v>463</v>
       </c>
       <c r="E75" t="s">
         <v>217</v>
       </c>
       <c r="F75" t="s">
-        <v>422</v>
+        <v>464</v>
       </c>
       <c r="H75" t="s">
         <v>219</v>
       </c>
-      <c r="J75">
-        <f t="shared" si="0"/>
-        <v>3958692308</v>
+      <c r="I75" t="s">
+        <v>461</v>
+      </c>
+      <c r="J75" t="s">
+        <v>461</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
-        <v>423</v>
+        <v>264</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>424</v>
+        <v>265</v>
       </c>
       <c r="C76" t="s">
-        <v>425</v>
+        <v>266</v>
       </c>
       <c r="D76" t="s">
-        <v>426</v>
-      </c>
-      <c r="E76" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="F76" t="s">
-        <v>427</v>
+        <v>268</v>
       </c>
       <c r="G76" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="H76" t="s">
-        <v>276</v>
-      </c>
-      <c r="J76" t="str">
-        <f t="shared" si="0"/>
-        <v>17841444720017694</v>
+        <v>537</v>
+      </c>
+      <c r="J76" t="s">
+        <v>264</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
-        <v>428</v>
+        <v>388</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>429</v>
-      </c>
-      <c r="C77" t="s">
-        <v>430</v>
+        <v>389</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>390</v>
       </c>
       <c r="D77" t="s">
-        <v>431</v>
+        <v>391</v>
       </c>
       <c r="E77" t="s">
-        <v>432</v>
+        <v>217</v>
       </c>
       <c r="F77" t="s">
-        <v>433</v>
+        <v>390</v>
       </c>
       <c r="H77" t="s">
-        <v>434</v>
-      </c>
-      <c r="I77" t="s">
-        <v>428</v>
-      </c>
-      <c r="J77" t="str">
-        <f t="shared" si="0"/>
-        <v>17841449463034944</v>
+        <v>219</v>
+      </c>
+      <c r="J77" t="s">
+        <v>388</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
-        <v>435</v>
+        <v>396</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>436</v>
+        <v>397</v>
       </c>
       <c r="C78" t="s">
-        <v>437</v>
+        <v>398</v>
       </c>
       <c r="D78" t="s">
-        <v>438</v>
-      </c>
-      <c r="E78" t="s">
-        <v>274</v>
+        <v>399</v>
       </c>
       <c r="F78" t="s">
-        <v>439</v>
+        <v>400</v>
       </c>
       <c r="G78" t="s">
-        <v>544</v>
+        <v>536</v>
       </c>
       <c r="H78" t="s">
-        <v>276</v>
-      </c>
-      <c r="I78" t="s">
-        <v>435</v>
+        <v>537</v>
       </c>
       <c r="J78" t="str">
-        <f t="shared" si="0"/>
-        <v>17841400778089100</v>
+        <f>A78</f>
+        <v>17841428945200784</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A79" s="1">
-        <v>7323028146</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>440</v>
+      <c r="A79" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>377</v>
       </c>
       <c r="C79" t="s">
-        <v>441</v>
+        <v>378</v>
       </c>
       <c r="D79" t="s">
-        <v>442</v>
+        <v>379</v>
       </c>
       <c r="E79" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="F79" t="s">
-        <v>443</v>
+        <v>378</v>
+      </c>
+      <c r="G79" t="s">
+        <v>536</v>
       </c>
       <c r="H79" t="s">
-        <v>219</v>
-      </c>
-      <c r="J79">
-        <f t="shared" si="0"/>
-        <v>7323028146</v>
+        <v>275</v>
+      </c>
+      <c r="J79" t="s">
+        <v>376</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
-        <v>444</v>
+        <v>401</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>445</v>
+        <v>402</v>
       </c>
       <c r="C80" t="s">
-        <v>446</v>
+        <v>403</v>
       </c>
       <c r="D80" t="s">
+        <v>404</v>
+      </c>
+      <c r="E80" t="s">
+        <v>217</v>
+      </c>
+      <c r="F80" t="s">
+        <v>405</v>
+      </c>
+      <c r="H80" t="s">
+        <v>219</v>
+      </c>
+      <c r="J80" t="str">
+        <f>A80</f>
+        <v>17841435108167586</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
         <v>447</v>
       </c>
-      <c r="E80" t="s">
-        <v>224</v>
-      </c>
-      <c r="F80" t="s">
+      <c r="C81" s="1" t="s">
         <v>448</v>
       </c>
-      <c r="G80" t="s">
-        <v>226</v>
-      </c>
-      <c r="H80" t="s">
-        <v>224</v>
-      </c>
-      <c r="I80" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A81" s="1" t="s">
+      <c r="D81" t="s">
         <v>449</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="E81" t="s">
+        <v>273</v>
+      </c>
+      <c r="F81" t="s">
         <v>450</v>
       </c>
-      <c r="C81" t="s">
-        <v>451</v>
-      </c>
-      <c r="D81" t="s">
-        <v>452</v>
-      </c>
-      <c r="E81" t="s">
-        <v>217</v>
-      </c>
-      <c r="F81" t="s">
-        <v>453</v>
-      </c>
       <c r="H81" t="s">
-        <v>219</v>
-      </c>
-      <c r="I81" t="s">
-        <v>454</v>
+        <v>275</v>
+      </c>
+      <c r="J81" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>455</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>456</v>
+      <c r="A82" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B82" s="3" t="s">
+        <v>357</v>
+      </c>
+      <c r="C82" t="s">
+        <v>358</v>
       </c>
       <c r="D82" t="s">
-        <v>457</v>
+        <v>359</v>
       </c>
       <c r="E82" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="F82" t="s">
-        <v>458</v>
+        <v>358</v>
+      </c>
+      <c r="G82" t="s">
+        <v>536</v>
       </c>
       <c r="H82" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J82" t="s">
-        <v>455</v>
+        <v>356</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
-        <v>459</v>
+        <v>415</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>460</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>461</v>
+        <v>416</v>
+      </c>
+      <c r="C83" t="s">
+        <v>417</v>
       </c>
       <c r="D83" t="s">
-        <v>462</v>
+        <v>418</v>
       </c>
       <c r="E83" t="s">
-        <v>217</v>
+        <v>273</v>
       </c>
       <c r="F83" t="s">
-        <v>463</v>
+        <v>419</v>
+      </c>
+      <c r="G83" t="s">
+        <v>536</v>
       </c>
       <c r="H83" t="s">
-        <v>219</v>
-      </c>
-      <c r="I83" t="s">
-        <v>464</v>
+        <v>275</v>
+      </c>
+      <c r="J83" t="str">
+        <f>A83</f>
+        <v>17841444720017694</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
-        <v>465</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>466</v>
+        <v>380</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="C84" s="5" t="s">
+        <v>382</v>
       </c>
       <c r="D84" t="s">
-        <v>467</v>
+        <v>383</v>
       </c>
       <c r="E84" t="s">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="F84" t="s">
-        <v>468</v>
+        <v>382</v>
       </c>
       <c r="H84" t="s">
-        <v>276</v>
-      </c>
-      <c r="I84" t="s">
-        <v>465</v>
+        <v>219</v>
       </c>
       <c r="J84" t="s">
-        <v>465</v>
+        <v>380</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
-        <v>469</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>470</v>
+        <v>420</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="C85" t="s">
+        <v>422</v>
       </c>
       <c r="D85" t="s">
-        <v>471</v>
+        <v>423</v>
       </c>
       <c r="E85" t="s">
+        <v>424</v>
+      </c>
+      <c r="F85" t="s">
+        <v>425</v>
+      </c>
+      <c r="H85" t="s">
+        <v>426</v>
+      </c>
+      <c r="I85" t="s">
+        <v>420</v>
+      </c>
+      <c r="J85" t="str">
+        <f>A85</f>
+        <v>17841449463034944</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
+        <v>457</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="D86" t="s">
+        <v>459</v>
+      </c>
+      <c r="E86" t="s">
+        <v>273</v>
+      </c>
+      <c r="F86" t="s">
+        <v>460</v>
+      </c>
+      <c r="H86" t="s">
+        <v>275</v>
+      </c>
+      <c r="I86" t="s">
+        <v>457</v>
+      </c>
+      <c r="J86" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="C87" t="s">
+        <v>515</v>
+      </c>
+      <c r="D87" s="8" t="s">
+        <v>516</v>
+      </c>
+      <c r="E87" t="s">
         <v>217</v>
       </c>
-      <c r="F85" t="s">
-        <v>472</v>
-      </c>
-      <c r="H85" t="s">
+      <c r="F87" t="s">
+        <v>517</v>
+      </c>
+      <c r="H87" t="s">
         <v>219</v>
       </c>
-      <c r="I85" t="s">
-        <v>469</v>
-      </c>
-      <c r="J85" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A86" t="str">
-        <f>C86</f>
-        <v>Bluey (Portugeuse)</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>473</v>
-      </c>
-      <c r="C86" t="s">
-        <v>474</v>
-      </c>
-      <c r="D86" t="s">
-        <v>475</v>
-      </c>
-      <c r="E86" t="s">
-        <v>274</v>
-      </c>
-      <c r="F86" t="s">
-        <v>476</v>
-      </c>
-      <c r="H86" t="s">
-        <v>276</v>
-      </c>
-      <c r="I86" t="s">
-        <v>473</v>
-      </c>
-      <c r="J86" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B87" t="s">
-        <v>477</v>
-      </c>
-      <c r="C87" t="s">
-        <v>478</v>
-      </c>
-      <c r="D87" t="s">
-        <v>479</v>
-      </c>
-      <c r="E87" t="s">
-        <v>274</v>
-      </c>
-      <c r="F87" t="s">
-        <v>480</v>
-      </c>
-      <c r="H87" t="s">
-        <v>276</v>
-      </c>
-      <c r="I87" t="s">
-        <v>477</v>
-      </c>
-      <c r="J87" t="s">
-        <v>477</v>
+      <c r="I87" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="J87" s="1" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A88" s="9">
-        <v>59656647810</v>
+      <c r="A88" s="11" t="s">
+        <v>492</v>
       </c>
       <c r="B88" s="1" t="s">
+        <v>493</v>
+      </c>
+      <c r="C88" s="11" t="s">
+        <v>494</v>
+      </c>
+      <c r="D88" t="s">
+        <v>495</v>
+      </c>
+      <c r="F88" t="s">
+        <v>496</v>
+      </c>
+      <c r="H88" t="s">
+        <v>497</v>
+      </c>
+      <c r="I88" s="11" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A89" s="11" t="s">
         <v>481</v>
       </c>
-      <c r="D88" s="10" t="s">
+      <c r="B89" s="1" t="s">
         <v>482</v>
       </c>
-      <c r="E88" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="F88" s="10" t="s">
+      <c r="C89" s="11" t="s">
         <v>483</v>
       </c>
-      <c r="H88" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="I88" s="9">
-        <v>59656647810</v>
-      </c>
-      <c r="J88" s="9">
-        <v>59656647810</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A89" s="9">
-        <v>50063441671</v>
-      </c>
-      <c r="B89" s="1" t="s">
+      <c r="D89" s="11" t="s">
         <v>484</v>
       </c>
-      <c r="D89" s="10" t="s">
+      <c r="E89" t="s">
+        <v>205</v>
+      </c>
+      <c r="F89" t="s">
         <v>485</v>
       </c>
-      <c r="E89" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="F89" s="10" t="s">
+      <c r="H89" t="s">
+        <v>207</v>
+      </c>
+      <c r="I89" s="11" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A90" s="11" t="s">
         <v>486</v>
       </c>
-      <c r="H89" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="I89" s="9">
-        <v>50063441671</v>
-      </c>
-      <c r="J89" s="9">
-        <v>50063441671</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A90" s="9">
-        <v>60242160822</v>
-      </c>
       <c r="B90" s="1" t="s">
-        <v>484</v>
-      </c>
-      <c r="D90" s="8" t="s">
         <v>487</v>
       </c>
-      <c r="E90" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="F90" s="10" t="s">
+      <c r="C90" s="11" t="s">
         <v>488</v>
       </c>
-      <c r="H90" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="I90" s="9">
-        <v>60242160822</v>
-      </c>
-      <c r="J90" s="9">
-        <v>60242160822</v>
+      <c r="D90" s="11" t="s">
+        <v>489</v>
+      </c>
+      <c r="F90" s="11" t="s">
+        <v>490</v>
+      </c>
+      <c r="H90" s="11" t="s">
+        <v>491</v>
+      </c>
+      <c r="I90" s="11" t="s">
+        <v>486</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A91" s="11" t="s">
-        <v>489</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>490</v>
-      </c>
-      <c r="C91" s="11" t="s">
-        <v>491</v>
-      </c>
-      <c r="D91" s="11" t="s">
-        <v>492</v>
-      </c>
-      <c r="E91" t="s">
-        <v>205</v>
-      </c>
-      <c r="F91" t="s">
-        <v>493</v>
+      <c r="A91" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="B91"/>
+      <c r="C91" t="s">
+        <v>526</v>
       </c>
       <c r="H91" t="s">
-        <v>207</v>
-      </c>
-      <c r="I91" s="11" t="s">
-        <v>489</v>
+        <v>527</v>
+      </c>
+      <c r="I91" s="1" t="s">
+        <v>525</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A92" s="11" t="s">
-        <v>494</v>
+      <c r="A92" s="1" t="s">
+        <v>451</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>495</v>
-      </c>
-      <c r="C92" s="11" t="s">
-        <v>496</v>
-      </c>
-      <c r="D92" s="11" t="s">
-        <v>497</v>
-      </c>
-      <c r="F92" s="11" t="s">
+        <v>452</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="D92" t="s">
+        <v>454</v>
+      </c>
+      <c r="E92" t="s">
+        <v>217</v>
+      </c>
+      <c r="F92" t="s">
+        <v>455</v>
+      </c>
+      <c r="H92" t="s">
+        <v>219</v>
+      </c>
+      <c r="I92" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="B93" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="C93" t="s">
+        <v>443</v>
+      </c>
+      <c r="D93" t="s">
+        <v>444</v>
+      </c>
+      <c r="E93" t="s">
+        <v>217</v>
+      </c>
+      <c r="F93" t="s">
+        <v>445</v>
+      </c>
+      <c r="H93" t="s">
+        <v>219</v>
+      </c>
+      <c r="I93" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A94" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D94" t="s">
+        <v>95</v>
+      </c>
+      <c r="E94" t="s">
+        <v>24</v>
+      </c>
+      <c r="F94" t="s">
+        <v>96</v>
+      </c>
+      <c r="H94" t="s">
+        <v>24</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
         <v>498</v>
       </c>
-      <c r="H92" s="11" t="s">
+      <c r="C95" t="s">
+        <v>498</v>
+      </c>
+      <c r="D95" t="s">
         <v>499</v>
       </c>
-      <c r="I92" s="11" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A93" s="11" t="s">
+      <c r="F95" t="s">
         <v>500</v>
       </c>
-      <c r="B93" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="C93" s="11" t="s">
-        <v>502</v>
-      </c>
-      <c r="D93" t="s">
-        <v>503</v>
-      </c>
-      <c r="F93" t="s">
-        <v>504</v>
-      </c>
-      <c r="H93" t="s">
-        <v>505</v>
-      </c>
-      <c r="I93" s="11" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A94" t="s">
-        <v>506</v>
-      </c>
-      <c r="C94" t="s">
-        <v>506</v>
-      </c>
-      <c r="D94" t="s">
-        <v>507</v>
-      </c>
-      <c r="F94" t="s">
-        <v>508</v>
-      </c>
-      <c r="H94" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A95" t="str">
-        <f>C95</f>
-        <v>Bluey (Castilian Spanish)</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>509</v>
-      </c>
-      <c r="C95" t="s">
-        <v>510</v>
-      </c>
-      <c r="D95" t="s">
-        <v>511</v>
-      </c>
-      <c r="F95" t="s">
-        <v>512</v>
-      </c>
       <c r="H95" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" t="str">
-        <f>C96</f>
-        <v>Bluey (German)</v>
-      </c>
-      <c r="B96" s="3" t="s">
-        <v>278</v>
+        <f t="shared" ref="A96:A103" si="0">C96</f>
+        <v>Bluey (Castilian Spanish)</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>501</v>
       </c>
       <c r="C96" t="s">
-        <v>513</v>
+        <v>502</v>
       </c>
       <c r="D96" t="s">
-        <v>514</v>
+        <v>503</v>
       </c>
       <c r="F96" t="s">
-        <v>515</v>
+        <v>504</v>
       </c>
       <c r="H96" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" t="str">
-        <f>C97</f>
-        <v>Bluey (Korea)</v>
-      </c>
-      <c r="B97" s="3" t="s">
-        <v>278</v>
+        <f t="shared" si="0"/>
+        <v>Bluey (Espanol)</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>501</v>
       </c>
       <c r="C97" t="s">
-        <v>516</v>
-      </c>
-      <c r="D97" t="s">
-        <v>517</v>
-      </c>
-      <c r="F97" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="H97" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" t="str">
-        <f>C98</f>
-        <v>Bluey (Japanese)</v>
-      </c>
-      <c r="B98" s="3" t="s">
-        <v>278</v>
+        <f t="shared" si="0"/>
+        <v>Bluey (French)</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>473</v>
       </c>
       <c r="C98" t="s">
-        <v>519</v>
-      </c>
-      <c r="D98" t="s">
-        <v>520</v>
-      </c>
-      <c r="F98" t="s">
-        <v>521</v>
+        <v>518</v>
       </c>
       <c r="H98" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A99" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>522</v>
+      <c r="A99" t="str">
+        <f t="shared" si="0"/>
+        <v>Bluey (German)</v>
+      </c>
+      <c r="B99" s="3" t="s">
+        <v>277</v>
       </c>
       <c r="C99" t="s">
-        <v>523</v>
-      </c>
-      <c r="D99" s="8" t="s">
-        <v>524</v>
-      </c>
-      <c r="E99" t="s">
-        <v>217</v>
+        <v>505</v>
+      </c>
+      <c r="D99" t="s">
+        <v>506</v>
       </c>
       <c r="F99" t="s">
-        <v>525</v>
+        <v>507</v>
       </c>
       <c r="H99" t="s">
-        <v>219</v>
-      </c>
-      <c r="I99" s="1" t="s">
-        <v>522</v>
-      </c>
-      <c r="J99" s="1" t="s">
-        <v>522</v>
+        <v>275</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" t="str">
-        <f>C100</f>
-        <v>Bluey (French)</v>
+        <f t="shared" si="0"/>
+        <v>Bluey (Italian)</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="C100" t="s">
-        <v>526</v>
+        <v>519</v>
       </c>
       <c r="H100" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" t="str">
-        <f>C101</f>
-        <v>Bluey (Italian)</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>484</v>
+        <f t="shared" si="0"/>
+        <v>Bluey (Japanese)</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>277</v>
       </c>
       <c r="C101" t="s">
-        <v>527</v>
+        <v>511</v>
+      </c>
+      <c r="D101" t="s">
+        <v>512</v>
+      </c>
+      <c r="F101" t="s">
+        <v>513</v>
       </c>
       <c r="H101" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" t="str">
-        <f>C102</f>
-        <v>Bluey (Espanol)</v>
-      </c>
-      <c r="B102" s="1" t="s">
+        <f t="shared" si="0"/>
+        <v>Bluey (Korea)</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C102" t="s">
+        <v>508</v>
+      </c>
+      <c r="D102" t="s">
         <v>509</v>
       </c>
-      <c r="C102" t="s">
-        <v>528</v>
+      <c r="F102" t="s">
+        <v>510</v>
       </c>
       <c r="H102" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>529</v>
-      </c>
-      <c r="B103" s="3" t="s">
-        <v>530</v>
+      <c r="A103" t="str">
+        <f t="shared" si="0"/>
+        <v>Bluey (Portugeuse)</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>465</v>
       </c>
       <c r="C103" t="s">
-        <v>531</v>
+        <v>466</v>
+      </c>
+      <c r="D103" t="s">
+        <v>467</v>
       </c>
       <c r="E103" t="s">
-        <v>224</v>
+        <v>273</v>
       </c>
       <c r="F103" t="s">
-        <v>532</v>
-      </c>
-      <c r="G103" t="s">
-        <v>544</v>
+        <v>468</v>
       </c>
       <c r="H103" t="s">
-        <v>224</v>
+        <v>275</v>
+      </c>
+      <c r="I103" t="s">
+        <v>465</v>
+      </c>
+      <c r="J103" t="s">
+        <v>465</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A104" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="B104"/>
+      <c r="A104" t="s">
+        <v>469</v>
+      </c>
+      <c r="B104" t="s">
+        <v>469</v>
+      </c>
       <c r="C104" t="s">
-        <v>534</v>
+        <v>470</v>
+      </c>
+      <c r="D104" t="s">
+        <v>471</v>
       </c>
       <c r="E104" t="s">
-        <v>535</v>
+        <v>273</v>
+      </c>
+      <c r="F104" t="s">
+        <v>472</v>
       </c>
       <c r="H104" t="s">
-        <v>535</v>
-      </c>
-      <c r="I104" s="1" t="s">
-        <v>533</v>
-      </c>
-      <c r="J104" s="1" t="s">
-        <v>533</v>
+        <v>275</v>
+      </c>
+      <c r="I104" t="s">
+        <v>469</v>
+      </c>
+      <c r="J104" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A105" s="1" t="s">
-        <v>536</v>
-      </c>
-      <c r="B105" s="3"/>
-      <c r="C105" s="12" t="s">
-        <v>537</v>
-      </c>
-      <c r="E105" t="s">
-        <v>219</v>
-      </c>
-      <c r="F105" t="s">
-        <v>538</v>
-      </c>
+      <c r="A105"/>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A106"/>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107"/>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108"/>
+      <c r="B108"/>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109"/>
+      <c r="B109"/>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110"/>
@@ -5030,51 +4972,47 @@
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A139"/>
-      <c r="B139"/>
+      <c r="B139" s="12"/>
+      <c r="C139" s="13"/>
+      <c r="I139" s="12"/>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A140"/>
-      <c r="B140"/>
+      <c r="B140" s="12"/>
+      <c r="C140" s="13"/>
+      <c r="I140" s="12"/>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A141"/>
-      <c r="B141" s="13"/>
-      <c r="C141" s="14"/>
-      <c r="I141" s="13"/>
+      <c r="B141"/>
+      <c r="C141" s="13"/>
+      <c r="I141" s="12"/>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A142"/>
-      <c r="B142" s="13"/>
-      <c r="C142" s="14"/>
-      <c r="I142" s="13"/>
+      <c r="C142" s="13"/>
+      <c r="I142" s="12"/>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A143"/>
-      <c r="B143"/>
-      <c r="C143" s="14"/>
-      <c r="I143" s="13"/>
+      <c r="C143" s="13"/>
+      <c r="I143" s="12"/>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A144"/>
-      <c r="C144" s="14"/>
-      <c r="I144" s="13"/>
-    </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A145"/>
-      <c r="C145" s="14"/>
-      <c r="I145" s="13"/>
-    </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A146"/>
-      <c r="C146" s="14"/>
-      <c r="I146" s="13"/>
+      <c r="C144" s="13"/>
+      <c r="I144" s="12"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J105" xr:uid="{CBB8FDA3-6C63-BA45-BC17-0CCC0291ABA7}"/>
+  <autoFilter ref="A1:J104" xr:uid="{CBB8FDA3-6C63-BA45-BC17-0CCC0291ABA7}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J104">
+      <sortCondition ref="A1:A104"/>
+    </sortState>
+  </autoFilter>
   <hyperlinks>
-    <hyperlink ref="D71" r:id="rId1" xr:uid="{DB7B27C7-1E96-8A49-8C39-B2888241DAAB}"/>
-    <hyperlink ref="D90" r:id="rId2" xr:uid="{332B75DD-7303-5D47-83A8-9DE375293A96}"/>
-    <hyperlink ref="D99" r:id="rId3" xr:uid="{CDC1F7C1-3AB9-3348-9253-85031F154076}"/>
+    <hyperlink ref="D27" r:id="rId1" xr:uid="{DB7B27C7-1E96-8A49-8C39-B2888241DAAB}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{332B75DD-7303-5D47-83A8-9DE375293A96}"/>
+    <hyperlink ref="D87" r:id="rId3" xr:uid="{CDC1F7C1-3AB9-3348-9253-85031F154076}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>